<commit_message>
Updated CHN_grids_kan10 model - 2026-02-19 21:44
</commit_message>
<xml_diff>
--- a/VerveStacks_CHN_grids_kan10/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_CHN_grids_kan10/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHN_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A5A39B8-91CF-48C8-A085-54F73CCF91A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B4E8C60-D6D1-4682-B2E1-A4A3F288A117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3308" yWindow="3308" windowWidth="21600" windowHeight="12682" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap" sheetId="56" r:id="rId1"/>
@@ -7206,7 +7206,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F64EC36C-07DC-4CA3-A585-CF4977EA42C1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84B9D91A-3F72-491D-AFF5-C2DE080BFDA5}">
   <dimension ref="B9:L305"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -39651,7 +39651,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AC86B6E-EA36-4D67-BD9C-AC897F02D263}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E02E9B5-BAC7-4C02-98E7-90DEA7929435}">
   <dimension ref="B9:H305"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated CHN_grids_kan10 model - 2026-02-20 00:58
</commit_message>
<xml_diff>
--- a/VerveStacks_CHN_grids_kan10/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_CHN_grids_kan10/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_CHN_grids_kan10\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B4E8C60-D6D1-4682-B2E1-A4A3F288A117}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ACEF50E3-CBD6-432A-9DC5-B86B803EF3E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7206,7 +7206,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84B9D91A-3F72-491D-AFF5-C2DE080BFDA5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{275622AE-9F8D-429A-9FE4-4C95C86E8C02}">
   <dimension ref="B9:L305"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -39651,7 +39651,7 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E02E9B5-BAC7-4C02-98E7-90DEA7929435}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FA35D30-09E1-43FB-BD58-FF0660B669DD}">
   <dimension ref="B9:H305"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>